<commit_message>
Agregar salidas del TP3
</commit_message>
<xml_diff>
--- a/TP3/salidas/tablas/TP3_Balance_Table_Train_2024_vs_Test_2025.xlsx
+++ b/TP3/salidas/tablas/TP3_Balance_Table_Train_2024_vs_Test_2025.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -727,56 +727,26 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>asalariado</t>
+          <t>tiene_cobertura_salud</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.6875</v>
+        <v>0.7438</v>
       </c>
       <c r="C11" t="n">
-        <v>0.6664</v>
+        <v>0.7348</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.0211</v>
+        <v>-0.008999999999999999</v>
       </c>
       <c r="E11" t="n">
-        <v>0.0007</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>***</t>
-        </is>
-      </c>
+        <v>0.1228</v>
+      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
         <v>11789</v>
       </c>
       <c r="H11" t="n">
-        <v>10849</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>tiene_cobertura_salud</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>0.7438</v>
-      </c>
-      <c r="C12" t="n">
-        <v>0.7348</v>
-      </c>
-      <c r="D12" t="n">
-        <v>-0.008999999999999999</v>
-      </c>
-      <c r="E12" t="n">
-        <v>0.1228</v>
-      </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="n">
-        <v>11789</v>
-      </c>
-      <c r="H12" t="n">
         <v>10849</v>
       </c>
     </row>

</xml_diff>